<commit_message>
repairing the dl runscripts
</commit_message>
<xml_diff>
--- a/benchmarking/analylsis/averages.xlsx
+++ b/benchmarking/analylsis/averages.xlsx
@@ -3,8 +3,10 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="wide" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="tall" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="exp1-wide" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="exp1-tall" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="exp2-wide" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="exp2-tall" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -12,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="21">
   <si>
     <t>MAPF</t>
   </si>
@@ -60,6 +62,21 @@
   </si>
   <si>
     <t>drive-hyper</t>
+  </si>
+  <si>
+    <t>compact-edge-functions</t>
+  </si>
+  <si>
+    <t>compact-subnodes</t>
+  </si>
+  <si>
+    <t>compact-hypergraph</t>
+  </si>
+  <si>
+    <t>compact-edge</t>
+  </si>
+  <si>
+    <t>compact-hyper</t>
   </si>
 </sst>
 </file>
@@ -179,6 +196,14 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -974,8 +999,8 @@
   <mergeCells count="4">
     <mergeCell ref="C1:H1"/>
     <mergeCell ref="I1:N1"/>
+    <mergeCell ref="O1:T1"/>
     <mergeCell ref="U1:Z1"/>
-    <mergeCell ref="O1:T1"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1716,4 +1741,1034 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C3" s="8">
+        <v>10.1503428571429</v>
+      </c>
+      <c r="D3" s="8">
+        <v>15.8772</v>
+      </c>
+      <c r="E3" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="F3" s="10">
+        <v>3054206.68571429</v>
+      </c>
+      <c r="G3" s="10">
+        <v>1069490.54285714</v>
+      </c>
+      <c r="H3" s="10">
+        <v>5185702.2</v>
+      </c>
+      <c r="I3" s="11">
+        <v>2.70914285714286</v>
+      </c>
+      <c r="J3" s="11">
+        <v>2.98214285714286</v>
+      </c>
+      <c r="K3" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="L3" s="13">
+        <v>549975.914285714</v>
+      </c>
+      <c r="M3" s="13">
+        <v>424274.071428571</v>
+      </c>
+      <c r="N3" s="13">
+        <v>1567199.45714286</v>
+      </c>
+      <c r="O3" s="8">
+        <v>9.42044285714286</v>
+      </c>
+      <c r="P3" s="8">
+        <v>14.1234428571429</v>
+      </c>
+      <c r="Q3" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="R3" s="10">
+        <v>2589443.81428571</v>
+      </c>
+      <c r="S3" s="10">
+        <v>958858.928571429</v>
+      </c>
+      <c r="T3" s="10">
+        <v>4242545.74285714</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C4" s="8">
+        <v>17.8334428571429</v>
+      </c>
+      <c r="D4" s="8">
+        <v>34.4610142857143</v>
+      </c>
+      <c r="E4" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="F4" s="10">
+        <v>5056109.52857143</v>
+      </c>
+      <c r="G4" s="10">
+        <v>1838336.37142857</v>
+      </c>
+      <c r="H4" s="10">
+        <v>8959021.1</v>
+      </c>
+      <c r="I4" s="11">
+        <v>4.5422</v>
+      </c>
+      <c r="J4" s="11">
+        <v>5.94577142857143</v>
+      </c>
+      <c r="K4" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="L4" s="13">
+        <v>962308.285714286</v>
+      </c>
+      <c r="M4" s="13">
+        <v>719000.542857143</v>
+      </c>
+      <c r="N4" s="13">
+        <v>2705885.2</v>
+      </c>
+      <c r="O4" s="8">
+        <v>16.3332714285714</v>
+      </c>
+      <c r="P4" s="8">
+        <v>40.0371285714286</v>
+      </c>
+      <c r="Q4" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="R4" s="10">
+        <v>4353679.12857143</v>
+      </c>
+      <c r="S4" s="10">
+        <v>1680912.32857143</v>
+      </c>
+      <c r="T4" s="10">
+        <v>7452656.44285714</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C5" s="8">
+        <v>26.4042428571429</v>
+      </c>
+      <c r="D5" s="8">
+        <v>79.4683857142857</v>
+      </c>
+      <c r="E5" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="F5" s="10">
+        <v>7153301.98571429</v>
+      </c>
+      <c r="G5" s="10">
+        <v>2654786.14285714</v>
+      </c>
+      <c r="H5" s="10">
+        <v>1.28759131E7</v>
+      </c>
+      <c r="I5" s="11">
+        <v>6.75228571428571</v>
+      </c>
+      <c r="J5" s="11">
+        <v>10.8462857142857</v>
+      </c>
+      <c r="K5" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="L5" s="13">
+        <v>1452521.32857143</v>
+      </c>
+      <c r="M5" s="13">
+        <v>1054568.51428571</v>
+      </c>
+      <c r="N5" s="13">
+        <v>4051061.24285714</v>
+      </c>
+      <c r="O5" s="8">
+        <v>23.9275</v>
+      </c>
+      <c r="P5" s="8">
+        <v>80.8897857142857</v>
+      </c>
+      <c r="Q5" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="R5" s="10">
+        <v>6132260.68571429</v>
+      </c>
+      <c r="S5" s="10">
+        <v>2408996.97142857</v>
+      </c>
+      <c r="T5" s="10">
+        <v>1.07226185142857E7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C6" s="8">
+        <v>34.0283142857143</v>
+      </c>
+      <c r="D6" s="8">
+        <v>134.0566</v>
+      </c>
+      <c r="E6" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="10">
+        <v>8979297.21428571</v>
+      </c>
+      <c r="G6" s="10">
+        <v>3258335.64285714</v>
+      </c>
+      <c r="H6" s="10">
+        <v>1.59369788571429E7</v>
+      </c>
+      <c r="I6" s="11">
+        <v>8.55904285714286</v>
+      </c>
+      <c r="J6" s="11">
+        <v>21.3990428571429</v>
+      </c>
+      <c r="K6" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="L6" s="13">
+        <v>1885057.95714286</v>
+      </c>
+      <c r="M6" s="13">
+        <v>1322523.3</v>
+      </c>
+      <c r="N6" s="13">
+        <v>5144477.72857143</v>
+      </c>
+      <c r="O6" s="8">
+        <v>30.1581</v>
+      </c>
+      <c r="P6" s="8">
+        <v>124.350528571429</v>
+      </c>
+      <c r="Q6" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="R6" s="10">
+        <v>7722279.85714286</v>
+      </c>
+      <c r="S6" s="10">
+        <v>2964259.91428571</v>
+      </c>
+      <c r="T6" s="10">
+        <v>1.32945689857143E7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C7" s="8">
+        <v>41.9537142857143</v>
+      </c>
+      <c r="D7" s="8">
+        <v>167.963</v>
+      </c>
+      <c r="E7" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="10">
+        <v>1.10377725571429E7</v>
+      </c>
+      <c r="G7" s="10">
+        <v>4007650.15714286</v>
+      </c>
+      <c r="H7" s="10">
+        <v>1.96620371714286E7</v>
+      </c>
+      <c r="I7" s="11">
+        <v>10.8055428571429</v>
+      </c>
+      <c r="J7" s="11">
+        <v>53.4901142857143</v>
+      </c>
+      <c r="K7" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="L7" s="13">
+        <v>2374802.78571429</v>
+      </c>
+      <c r="M7" s="13">
+        <v>1600442.51428571</v>
+      </c>
+      <c r="N7" s="13">
+        <v>6313807.1</v>
+      </c>
+      <c r="O7" s="8">
+        <v>37.4066</v>
+      </c>
+      <c r="P7" s="8">
+        <v>291.815885714286</v>
+      </c>
+      <c r="Q7" s="9">
+        <v>1.0</v>
+      </c>
+      <c r="R7" s="10">
+        <v>9498969.77142857</v>
+      </c>
+      <c r="S7" s="10">
+        <v>3641839.51428571</v>
+      </c>
+      <c r="T7" s="10">
+        <v>1.64266229142857E7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="C8" s="8">
+        <v>50.9206</v>
+      </c>
+      <c r="D8" s="8">
+        <v>263.9376</v>
+      </c>
+      <c r="E8" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="10">
+        <v>1.29265923E7</v>
+      </c>
+      <c r="G8" s="10">
+        <v>4706535.0</v>
+      </c>
+      <c r="H8" s="10">
+        <v>2.30731206E7</v>
+      </c>
+      <c r="I8" s="11">
+        <v>12.9696</v>
+      </c>
+      <c r="J8" s="11">
+        <v>62.9706</v>
+      </c>
+      <c r="K8" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="L8" s="13">
+        <v>2794790.8</v>
+      </c>
+      <c r="M8" s="13">
+        <v>1879691.6</v>
+      </c>
+      <c r="N8" s="13">
+        <v>7425011.9</v>
+      </c>
+      <c r="O8" s="8">
+        <v>44.0125</v>
+      </c>
+      <c r="P8" s="8">
+        <v>511.0645</v>
+      </c>
+      <c r="Q8" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="R8" s="10">
+        <v>1.11387017E7</v>
+      </c>
+      <c r="S8" s="10">
+        <v>4281979.9</v>
+      </c>
+      <c r="T8" s="10">
+        <v>1.93011785E7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="I1:N1"/>
+    <mergeCell ref="O1:T1"/>
+  </mergeCells>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="3" max="3" width="15.5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="B2" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="11">
+        <v>10.1503428571429</v>
+      </c>
+      <c r="E2" s="11">
+        <v>15.8772</v>
+      </c>
+      <c r="F2" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G2" s="13">
+        <v>3054206.68571429</v>
+      </c>
+      <c r="H2" s="13">
+        <v>1069490.54285714</v>
+      </c>
+      <c r="I2" s="13">
+        <v>5185702.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="B3" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="11">
+        <v>17.8334428571429</v>
+      </c>
+      <c r="E3" s="11">
+        <v>34.4610142857143</v>
+      </c>
+      <c r="F3" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G3" s="13">
+        <v>5056109.52857143</v>
+      </c>
+      <c r="H3" s="13">
+        <v>1838336.37142857</v>
+      </c>
+      <c r="I3" s="13">
+        <v>8959021.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="B4" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="11">
+        <v>26.4042428571429</v>
+      </c>
+      <c r="E4" s="11">
+        <v>79.4683857142857</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G4" s="13">
+        <v>7153301.98571429</v>
+      </c>
+      <c r="H4" s="13">
+        <v>2654786.14285714</v>
+      </c>
+      <c r="I4" s="13">
+        <v>1.28759131E7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="B5" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="11">
+        <v>34.0283142857143</v>
+      </c>
+      <c r="E5" s="11">
+        <v>134.0566</v>
+      </c>
+      <c r="F5" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G5" s="13">
+        <v>8979297.21428571</v>
+      </c>
+      <c r="H5" s="13">
+        <v>3258335.64285714</v>
+      </c>
+      <c r="I5" s="13">
+        <v>1.59369788571429E7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="B6" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="11">
+        <v>41.9537142857143</v>
+      </c>
+      <c r="E6" s="11">
+        <v>167.963</v>
+      </c>
+      <c r="F6" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G6" s="13">
+        <v>1.10377725571429E7</v>
+      </c>
+      <c r="H6" s="13">
+        <v>4007650.15714286</v>
+      </c>
+      <c r="I6" s="13">
+        <v>1.96620371714286E7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="B7" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="11">
+        <v>50.9206</v>
+      </c>
+      <c r="E7" s="11">
+        <v>263.9376</v>
+      </c>
+      <c r="F7" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G7" s="13">
+        <v>1.29265923E7</v>
+      </c>
+      <c r="H7" s="13">
+        <v>4706535.0</v>
+      </c>
+      <c r="I7" s="13">
+        <v>2.30731206E7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="B8" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="11">
+        <v>2.70914285714286</v>
+      </c>
+      <c r="E8" s="11">
+        <v>2.98214285714286</v>
+      </c>
+      <c r="F8" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G8" s="13">
+        <v>549975.914285714</v>
+      </c>
+      <c r="H8" s="13">
+        <v>424274.071428571</v>
+      </c>
+      <c r="I8" s="13">
+        <v>1567199.45714286</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="B9" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="11">
+        <v>4.5422</v>
+      </c>
+      <c r="E9" s="11">
+        <v>5.94577142857143</v>
+      </c>
+      <c r="F9" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G9" s="13">
+        <v>962308.285714286</v>
+      </c>
+      <c r="H9" s="13">
+        <v>719000.542857143</v>
+      </c>
+      <c r="I9" s="13">
+        <v>2705885.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="B10" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="11">
+        <v>6.75228571428571</v>
+      </c>
+      <c r="E10" s="11">
+        <v>10.8462857142857</v>
+      </c>
+      <c r="F10" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G10" s="13">
+        <v>1452521.32857143</v>
+      </c>
+      <c r="H10" s="13">
+        <v>1054568.51428571</v>
+      </c>
+      <c r="I10" s="13">
+        <v>4051061.24285714</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="B11" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="11">
+        <v>8.55904285714286</v>
+      </c>
+      <c r="E11" s="11">
+        <v>21.3990428571429</v>
+      </c>
+      <c r="F11" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G11" s="13">
+        <v>1885057.95714286</v>
+      </c>
+      <c r="H11" s="13">
+        <v>1322523.3</v>
+      </c>
+      <c r="I11" s="13">
+        <v>5144477.72857143</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="B12" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="11">
+        <v>10.8055428571429</v>
+      </c>
+      <c r="E12" s="11">
+        <v>53.4901142857143</v>
+      </c>
+      <c r="F12" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G12" s="13">
+        <v>2374802.78571429</v>
+      </c>
+      <c r="H12" s="13">
+        <v>1600442.51428571</v>
+      </c>
+      <c r="I12" s="13">
+        <v>6313807.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="B13" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="11">
+        <v>12.9696</v>
+      </c>
+      <c r="E13" s="11">
+        <v>62.9706</v>
+      </c>
+      <c r="F13" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G13" s="13">
+        <v>2794790.8</v>
+      </c>
+      <c r="H13" s="13">
+        <v>1879691.6</v>
+      </c>
+      <c r="I13" s="13">
+        <v>7425011.9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="B14" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="11">
+        <v>9.42044285714286</v>
+      </c>
+      <c r="E14" s="11">
+        <v>14.1234428571429</v>
+      </c>
+      <c r="F14" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G14" s="13">
+        <v>2589443.81428571</v>
+      </c>
+      <c r="H14" s="13">
+        <v>958858.928571429</v>
+      </c>
+      <c r="I14" s="13">
+        <v>4242545.74285714</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="B15" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="11">
+        <v>16.3332714285714</v>
+      </c>
+      <c r="E15" s="11">
+        <v>40.0371285714286</v>
+      </c>
+      <c r="F15" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G15" s="13">
+        <v>4353679.12857143</v>
+      </c>
+      <c r="H15" s="13">
+        <v>1680912.32857143</v>
+      </c>
+      <c r="I15" s="13">
+        <v>7452656.44285714</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="B16" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="11">
+        <v>23.9275</v>
+      </c>
+      <c r="E16" s="11">
+        <v>80.8897857142857</v>
+      </c>
+      <c r="F16" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G16" s="13">
+        <v>6132260.68571429</v>
+      </c>
+      <c r="H16" s="13">
+        <v>2408996.97142857</v>
+      </c>
+      <c r="I16" s="13">
+        <v>1.07226185142857E7</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="B17" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="11">
+        <v>30.1581</v>
+      </c>
+      <c r="E17" s="11">
+        <v>124.350528571429</v>
+      </c>
+      <c r="F17" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G17" s="13">
+        <v>7722279.85714286</v>
+      </c>
+      <c r="H17" s="13">
+        <v>2964259.91428571</v>
+      </c>
+      <c r="I17" s="13">
+        <v>1.32945689857143E7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="B18" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="11">
+        <v>37.4066</v>
+      </c>
+      <c r="E18" s="11">
+        <v>291.815885714286</v>
+      </c>
+      <c r="F18" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G18" s="13">
+        <v>9498969.77142857</v>
+      </c>
+      <c r="H18" s="13">
+        <v>3641839.51428571</v>
+      </c>
+      <c r="I18" s="13">
+        <v>1.64266229142857E7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="B19" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="11">
+        <v>44.0125</v>
+      </c>
+      <c r="E19" s="11">
+        <v>511.0645</v>
+      </c>
+      <c r="F19" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G19" s="13">
+        <v>1.11387017E7</v>
+      </c>
+      <c r="H19" s="13">
+        <v>4281979.9</v>
+      </c>
+      <c r="I19" s="13">
+        <v>1.93011785E7</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>